<commit_message>
chore: update tire inventory data
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="D4" s="0">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E4" s="0">
         <v>4</v>
@@ -482,7 +482,7 @@
         <v>3</v>
       </c>
       <c r="G4" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H4" s="1">
         <v>230</v>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D6" s="0">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E6" s="0">
         <v>4</v>
@@ -546,7 +546,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="0">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H6" s="1">
         <v>200</v>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D10" s="0">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E10" s="0">
         <v>4</v>
@@ -674,7 +674,7 @@
         <v>7</v>
       </c>
       <c r="G10" s="0">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H10" s="1">
         <v>270</v>
@@ -697,10 +697,10 @@
         </is>
       </c>
       <c r="D11" s="0">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E11" s="0">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F11" s="0">
         <v>0</v>
@@ -729,10 +729,10 @@
         </is>
       </c>
       <c r="D12" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E12" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" s="0">
         <v>18</v>
@@ -764,13 +764,13 @@
         <v>3</v>
       </c>
       <c r="E13" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F13" s="0">
         <v>0</v>
       </c>
       <c r="G13" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H13" s="1">
         <v>230</v>
@@ -921,10 +921,10 @@
         </is>
       </c>
       <c r="D18" s="0">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E18" s="0">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F18" s="0">
         <v>60</v>
@@ -953,10 +953,10 @@
         </is>
       </c>
       <c r="D19" s="0">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E19" s="0">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F19" s="0">
         <v>0</v>
@@ -1040,60 +1040,60 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>WESTLAKE</t>
+          <t>MATADOR</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>WL175/70R14</t>
+          <t>MT175/70R14</t>
         </is>
       </c>
       <c r="D22" s="0">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="E22" s="0">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F22" s="0">
         <v>0</v>
       </c>
       <c r="G22" s="0">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H22" s="1">
-        <v>200</v>
+        <v>230</v>
       </c>
     </row>
     <row outlineLevel="0" r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>185/55R15</t>
+          <t>175/70R14</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>BRIDGESTONE</t>
+          <t>WESTLAKE</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>BR185/55R15</t>
+          <t>WL175/70R14</t>
         </is>
       </c>
       <c r="D23" s="0">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="E23" s="0">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="F23" s="0">
         <v>0</v>
       </c>
       <c r="G23" s="0">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H23" s="1">
-        <v>370</v>
+        <v>200</v>
       </c>
     </row>
     <row outlineLevel="0" r="24">
@@ -1104,28 +1104,28 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>BRIDGESTONE</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>GD185/55R15</t>
+          <t>BR185/55R15</t>
         </is>
       </c>
       <c r="D24" s="0">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="E24" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F24" s="0">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="G24" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H24" s="1">
-        <v>340</v>
+        <v>370</v>
       </c>
     </row>
     <row outlineLevel="0" r="25">
@@ -1136,28 +1136,28 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>RD185/55R15</t>
+          <t>GD185/55R15</t>
         </is>
       </c>
       <c r="D25" s="0">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="E25" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F25" s="0">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="G25" s="0">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H25" s="1">
-        <v>270</v>
+        <v>340</v>
       </c>
     </row>
     <row outlineLevel="0" r="26">
@@ -1264,28 +1264,28 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>MATADOR</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>RD185/60R15</t>
+          <t>MT185/60R15</t>
         </is>
       </c>
       <c r="D29" s="0">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E29" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F29" s="0">
         <v>0</v>
       </c>
       <c r="G29" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H29" s="1">
-        <v>230</v>
+        <v>280</v>
       </c>
     </row>
     <row outlineLevel="0" r="30">
@@ -1296,25 +1296,25 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>WESTLAKE</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>WL185/60R15</t>
+          <t>RD185/60R15</t>
         </is>
       </c>
       <c r="D30" s="0">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E30" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" s="0">
         <v>0</v>
       </c>
       <c r="G30" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H30" s="1">
         <v>230</v>
@@ -1323,97 +1323,97 @@
     <row outlineLevel="0" r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>185/60R16</t>
+          <t>185/60R15</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>WESTLAKE</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>GD185/60R16</t>
+          <t>WL185/60R15</t>
         </is>
       </c>
       <c r="D31" s="0">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E31" s="0">
         <v>4</v>
       </c>
       <c r="F31" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G31" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H31" s="1">
-        <v>420</v>
+        <v>230</v>
       </c>
     </row>
     <row outlineLevel="0" r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>185/65R14</t>
+          <t>185/60R16</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>RD185/65R14</t>
+          <t>GD185/60R16</t>
         </is>
       </c>
       <c r="D32" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E32" s="0">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F32" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="0">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H32" s="1">
-        <v>200</v>
+        <v>420</v>
       </c>
     </row>
     <row outlineLevel="0" r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>185/65R15</t>
+          <t>185/65R14</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>CONTINENTAL</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>CT185/65R15</t>
+          <t>RD185/65R14</t>
         </is>
       </c>
       <c r="D33" s="0">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E33" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" s="0">
         <v>0</v>
       </c>
       <c r="G33" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H33" s="1">
-        <v>400</v>
+        <v>200</v>
       </c>
     </row>
     <row outlineLevel="0" r="34">
@@ -1424,28 +1424,28 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>DOUBLESTAR</t>
+          <t>CONTINENTAL</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>DS185/65R15</t>
+          <t>CT185/65R15</t>
         </is>
       </c>
       <c r="D34" s="0">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E34" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F34" s="0">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G34" s="0">
         <v>0</v>
       </c>
       <c r="H34" s="1">
-        <v>210</v>
+        <v>400</v>
       </c>
     </row>
     <row outlineLevel="0" r="35">
@@ -1456,28 +1456,28 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>FULDA</t>
+          <t>DOUBLESTAR</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>FL185/65R15</t>
+          <t>DS185/65R15</t>
         </is>
       </c>
       <c r="D35" s="0">
-        <v>136</v>
+        <v>7</v>
       </c>
       <c r="E35" s="0">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F35" s="0">
-        <v>109</v>
+        <v>5</v>
       </c>
       <c r="G35" s="0">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H35" s="1">
-        <v>245</v>
+        <v>210</v>
       </c>
     </row>
     <row outlineLevel="0" r="36">
@@ -1488,28 +1488,28 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>GOODRIDE</t>
+          <t>FULDA</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>GR185/65R15</t>
+          <t>FL185/65R15</t>
         </is>
       </c>
       <c r="D36" s="0">
+        <v>136</v>
+      </c>
+      <c r="E36" s="0">
+        <v>16</v>
+      </c>
+      <c r="F36" s="0">
+        <v>109</v>
+      </c>
+      <c r="G36" s="0">
         <v>11</v>
       </c>
-      <c r="E36" s="0">
-        <v>4</v>
-      </c>
-      <c r="F36" s="0">
-        <v>3</v>
-      </c>
-      <c r="G36" s="0">
-        <v>4</v>
-      </c>
       <c r="H36" s="1">
-        <v>230</v>
+        <v>245</v>
       </c>
     </row>
     <row outlineLevel="0" r="37">
@@ -1520,28 +1520,28 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>GOODRIDE</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>GD185/65R15</t>
+          <t>GR185/65R15</t>
         </is>
       </c>
       <c r="D37" s="0">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="E37" s="0">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F37" s="0">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="G37" s="0">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H37" s="1">
-        <v>260</v>
+        <v>230</v>
       </c>
     </row>
     <row outlineLevel="0" r="38">
@@ -1552,28 +1552,28 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>HK185/65R15</t>
+          <t>GD185/65R15</t>
         </is>
       </c>
       <c r="D38" s="0">
-        <v>5</v>
+        <v>67</v>
       </c>
       <c r="E38" s="0">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="F38" s="0">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="G38" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H38" s="1">
-        <v>250</v>
+        <v>260</v>
       </c>
     </row>
     <row outlineLevel="0" r="39">
@@ -1584,16 +1584,16 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>LUFEN</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>LF185/65R15</t>
+          <t>HK185/65R15</t>
         </is>
       </c>
       <c r="D39" s="0">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E39" s="0">
         <v>4</v>
@@ -1602,7 +1602,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39" s="1">
         <v>250</v>
@@ -1616,28 +1616,28 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>LUFEN</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>RD185/65R15</t>
+          <t>LF185/65R15</t>
         </is>
       </c>
       <c r="D40" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E40" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F40" s="0">
         <v>0</v>
       </c>
       <c r="G40" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H40" s="1">
-        <v>200</v>
+        <v>250</v>
       </c>
     </row>
     <row outlineLevel="0" r="41">
@@ -1648,28 +1648,28 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>SEMPERIT</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>SP185/65R15</t>
+          <t>RD185/65R15</t>
         </is>
       </c>
       <c r="D41" s="0">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E41" s="0">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F41" s="0">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G41" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H41" s="1">
-        <v>250</v>
+        <v>200</v>
       </c>
     </row>
     <row outlineLevel="0" r="42">
@@ -1680,60 +1680,60 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>WESTLAKE</t>
+          <t>SEMPERIT</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>WL185/65R15</t>
+          <t>SP185/65R15</t>
         </is>
       </c>
       <c r="D42" s="0">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="E42" s="0">
-        <v>86</v>
+        <v>5</v>
       </c>
       <c r="F42" s="0">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G42" s="0">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H42" s="1">
-        <v>220</v>
+        <v>250</v>
       </c>
     </row>
     <row outlineLevel="0" r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>185/70R14</t>
+          <t>185/65R15</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>WESTLAKE</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>RD185/70R14</t>
+          <t>WL185/65R15</t>
         </is>
       </c>
       <c r="D43" s="0">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="E43" s="0">
-        <v>1</v>
+        <v>86</v>
       </c>
       <c r="F43" s="0">
         <v>0</v>
       </c>
       <c r="G43" s="0">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H43" s="1">
-        <v>230</v>
+        <v>220</v>
       </c>
     </row>
     <row outlineLevel="0" r="44">
@@ -1744,28 +1744,28 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>SEMPERIT</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>SP185/70R14</t>
+          <t>RD185/70R14</t>
         </is>
       </c>
       <c r="D44" s="0">
         <v>2</v>
       </c>
       <c r="E44" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" s="0">
         <v>0</v>
       </c>
       <c r="G44" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H44" s="1">
-        <v>280</v>
+        <v>230</v>
       </c>
     </row>
     <row outlineLevel="0" r="45">
@@ -1776,60 +1776,60 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>WESTLAKE</t>
+          <t>SEMPERIT</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>WL185/70R14</t>
+          <t>SP185/70R14</t>
         </is>
       </c>
       <c r="D45" s="0">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E45" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F45" s="0">
         <v>0</v>
       </c>
       <c r="G45" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H45" s="1">
-        <v>220</v>
+        <v>280</v>
       </c>
     </row>
     <row outlineLevel="0" r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t>195/50R15</t>
+          <t>185/70R14</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>WESTLAKE</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>GD195/50R15</t>
+          <t>WL185/70R14</t>
         </is>
       </c>
       <c r="D46" s="0">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E46" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F46" s="0">
         <v>0</v>
       </c>
       <c r="G46" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H46" s="1">
-        <v>290</v>
+        <v>220</v>
       </c>
     </row>
     <row outlineLevel="0" r="47">
@@ -1840,28 +1840,28 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>SEMPERIT</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t>SP195/50R15</t>
+          <t>GD195/50R15</t>
         </is>
       </c>
       <c r="D47" s="0">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="E47" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F47" s="0">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G47" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H47" s="1">
-        <v>260</v>
+        <v>290</v>
       </c>
     </row>
     <row outlineLevel="0" r="48">
@@ -1872,66 +1872,66 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>WESTLAKE</t>
+          <t>SEMPERIT</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>WL195/50R15</t>
+          <t>SP195/50R15</t>
         </is>
       </c>
       <c r="D48" s="0">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E48" s="0">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F48" s="0">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G48" s="0">
         <v>4</v>
       </c>
       <c r="H48" s="1">
-        <v>225</v>
+        <v>260</v>
       </c>
     </row>
     <row outlineLevel="0" r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t>195/50R16</t>
+          <t>195/50R15</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>WESTLAKE</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>GD195/50R16</t>
+          <t>WL195/50R15</t>
         </is>
       </c>
       <c r="D49" s="0">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E49" s="0">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F49" s="0">
         <v>0</v>
       </c>
       <c r="G49" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H49" s="1">
-        <v>330</v>
+        <v>225</v>
       </c>
     </row>
     <row outlineLevel="0" r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t>195/55R16</t>
+          <t>195/50R16</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
@@ -1941,23 +1941,23 @@
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t>GD195/55R16</t>
+          <t>GD195/50R16</t>
         </is>
       </c>
       <c r="D50" s="0">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E50" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F50" s="0">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G50" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H50" s="1">
-        <v>350</v>
+        <v>330</v>
       </c>
     </row>
     <row outlineLevel="0" r="51">
@@ -1968,28 +1968,28 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t>HK195/55R16</t>
+          <t>GD195/55R16</t>
         </is>
       </c>
       <c r="D51" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E51" s="0">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F51" s="0">
         <v>13</v>
       </c>
       <c r="G51" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H51" s="1">
-        <v>290</v>
+        <v>350</v>
       </c>
     </row>
     <row outlineLevel="0" r="52">
@@ -2000,28 +2000,28 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>LASSA</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>LS195/55R16</t>
+          <t>HK195/55R16</t>
         </is>
       </c>
       <c r="D52" s="0">
+        <v>16</v>
+      </c>
+      <c r="E52" s="0">
+        <v>0</v>
+      </c>
+      <c r="F52" s="0">
+        <v>13</v>
+      </c>
+      <c r="G52" s="0">
         <v>3</v>
       </c>
-      <c r="E52" s="0">
-        <v>3</v>
-      </c>
-      <c r="F52" s="0">
-        <v>0</v>
-      </c>
-      <c r="G52" s="0">
-        <v>0</v>
-      </c>
       <c r="H52" s="1">
-        <v>280</v>
+        <v>290</v>
       </c>
     </row>
     <row outlineLevel="0" r="53">
@@ -2032,19 +2032,19 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>NEXEN</t>
+          <t>LASSA</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>NX195/55R16</t>
+          <t>LS195/55R16</t>
         </is>
       </c>
       <c r="D53" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E53" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F53" s="0">
         <v>0</v>
@@ -2053,7 +2053,7 @@
         <v>0</v>
       </c>
       <c r="H53" s="1">
-        <v>300</v>
+        <v>280</v>
       </c>
     </row>
     <row outlineLevel="0" r="54">
@@ -2064,92 +2064,92 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>NEXEN</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>RD195/55R16</t>
+          <t>NX195/55R16</t>
         </is>
       </c>
       <c r="D54" s="0">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E54" s="0">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F54" s="0">
         <v>0</v>
       </c>
       <c r="G54" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H54" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row outlineLevel="0" r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t>195/60R16</t>
+          <t>195/55R16</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>GD195/60R16</t>
+          <t>RD195/55R16</t>
         </is>
       </c>
       <c r="D55" s="0">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E55" s="0">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F55" s="0">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="G55" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H55" s="1">
-        <v>355</v>
+        <v>250</v>
       </c>
     </row>
     <row outlineLevel="0" r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t>195/65R15</t>
+          <t>195/60R16</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>DOUBLESTAR</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>DS195/65R15</t>
+          <t>GD195/60R16</t>
         </is>
       </c>
       <c r="D56" s="0">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="E56" s="0">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F56" s="0">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="G56" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H56" s="1">
-        <v>230</v>
+        <v>355</v>
       </c>
     </row>
     <row outlineLevel="0" r="57">
@@ -2160,22 +2160,22 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>GOODRIDE</t>
+          <t>DOUBLESTAR</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>GR195/65R15</t>
+          <t>DS195/65R15</t>
         </is>
       </c>
       <c r="D57" s="0">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E57" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F57" s="0">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G57" s="0">
         <v>0</v>
@@ -2192,28 +2192,28 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODRIDE</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>HK195/65R15</t>
+          <t>GR195/65R15</t>
         </is>
       </c>
       <c r="D58" s="0">
         <v>4</v>
       </c>
       <c r="E58" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F58" s="0">
         <v>0</v>
       </c>
       <c r="G58" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H58" s="1">
-        <v>260</v>
+        <v>230</v>
       </c>
     </row>
     <row outlineLevel="0" r="59">
@@ -2224,28 +2224,28 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>LASSA</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t>LS195/65R15</t>
+          <t>HK195/65R15</t>
         </is>
       </c>
       <c r="D59" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E59" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F59" s="0">
         <v>0</v>
       </c>
       <c r="G59" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H59" s="1">
-        <v>250</v>
+        <v>260</v>
       </c>
     </row>
     <row outlineLevel="0" r="60">
@@ -2256,19 +2256,19 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>NEXEN</t>
+          <t>LASSA</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>NX195/65R15</t>
+          <t>LS195/65R15</t>
         </is>
       </c>
       <c r="D60" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E60" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" s="0">
         <v>0</v>
@@ -2277,7 +2277,7 @@
         <v>0</v>
       </c>
       <c r="H60" s="1">
-        <v>230</v>
+        <v>250</v>
       </c>
     </row>
     <row outlineLevel="0" r="61">
@@ -2288,25 +2288,25 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>NEXEN</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t>RD195/65R15</t>
+          <t>NX195/65R15</t>
         </is>
       </c>
       <c r="D61" s="0">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E61" s="0">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F61" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G61" s="0">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H61" s="1">
         <v>230</v>
@@ -2320,140 +2320,140 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>SEMPERIT</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t>SP195/65R15</t>
+          <t>RD195/65R15</t>
         </is>
       </c>
       <c r="D62" s="0">
-        <v>96</v>
+        <v>15</v>
       </c>
       <c r="E62" s="0">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F62" s="0">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="G62" s="0">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H62" s="1">
-        <v>250</v>
+        <v>230</v>
       </c>
     </row>
     <row outlineLevel="0" r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t>195/70R15C</t>
+          <t>195/65R15</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>DAYTON</t>
+          <t>SEMPERIT</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t>DT195/70R15C</t>
+          <t>SP195/65R15</t>
         </is>
       </c>
       <c r="D63" s="0">
-        <v>2</v>
+        <v>96</v>
       </c>
       <c r="E63" s="0">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F63" s="0">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="G63" s="0">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H63" s="1">
-        <v>280</v>
+        <v>250</v>
       </c>
     </row>
     <row outlineLevel="0" r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t>195/75R16C</t>
+          <t>195/70R15C</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>GOODRIDE</t>
+          <t>DAYTON</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t>GR195/75R16C</t>
+          <t>DT195/70R15C</t>
         </is>
       </c>
       <c r="D64" s="0">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E64" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F64" s="0">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G64" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H64" s="1">
-        <v>350</v>
+        <v>280</v>
       </c>
     </row>
     <row outlineLevel="0" r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t>195R15C</t>
+          <t>195/75R16C</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>GOODRIDE</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t>RD195R15C</t>
+          <t>GR195/75R16C</t>
         </is>
       </c>
       <c r="D65" s="0">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E65" s="0">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F65" s="0">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G65" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H65" s="1">
-        <v>250</v>
+        <v>350</v>
       </c>
     </row>
     <row outlineLevel="0" r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t>205/45R17</t>
+          <t>195R15C</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>CONTINENTAL</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t>CT205/45R17</t>
+          <t>RD195R15C</t>
         </is>
       </c>
       <c r="D66" s="0">
@@ -2469,7 +2469,7 @@
         <v>0</v>
       </c>
       <c r="H66" s="1">
-        <v>550</v>
+        <v>250</v>
       </c>
     </row>
     <row outlineLevel="0" r="67">
@@ -2480,28 +2480,28 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>FULDA</t>
+          <t>CONTINENTAL</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t>FL205/45R17</t>
+          <t>CT205/45R17</t>
         </is>
       </c>
       <c r="D67" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E67" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F67" s="0">
         <v>0</v>
       </c>
       <c r="G67" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H67" s="1">
-        <v>380</v>
+        <v>550</v>
       </c>
     </row>
     <row outlineLevel="0" r="68">
@@ -2512,28 +2512,28 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>GOODRIDE</t>
+          <t>FULDA</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t>GR205/45R17</t>
+          <t>FL205/45R17</t>
         </is>
       </c>
       <c r="D68" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E68" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F68" s="0">
         <v>0</v>
       </c>
       <c r="G68" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H68" s="1">
-        <v>300</v>
+        <v>380</v>
       </c>
     </row>
     <row outlineLevel="0" r="69">
@@ -2544,28 +2544,28 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>GOODRIDE</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t>GD205/45R17</t>
+          <t>GR205/45R17</t>
         </is>
       </c>
       <c r="D69" s="0">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E69" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F69" s="0">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G69" s="0">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H69" s="1">
-        <v>450</v>
+        <v>300</v>
       </c>
     </row>
     <row outlineLevel="0" r="70">
@@ -2576,28 +2576,28 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>NEXEN</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t>NX205/45R17</t>
+          <t>GD205/45R17</t>
         </is>
       </c>
       <c r="D70" s="0">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E70" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F70" s="0">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G70" s="0">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H70" s="1">
-        <v>380</v>
+        <v>450</v>
       </c>
     </row>
     <row outlineLevel="0" r="71">
@@ -2608,83 +2608,83 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>NEXEN</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
         <is>
-          <t>RD205/45R17</t>
+          <t>NX205/45R17</t>
         </is>
       </c>
       <c r="D71" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F71" s="0">
         <v>0</v>
       </c>
       <c r="G71" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H71" s="1">
-        <v>300</v>
+        <v>380</v>
       </c>
     </row>
     <row outlineLevel="0" r="72">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t>205/50R17</t>
+          <t>205/45R17</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>CONTINENTAL</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
         <is>
-          <t>CT205/50R17</t>
+          <t>RD205/45R17</t>
         </is>
       </c>
       <c r="D72" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E72" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F72" s="0">
         <v>0</v>
       </c>
       <c r="G72" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H72" s="1">
-        <v>450</v>
+        <v>300</v>
       </c>
     </row>
     <row outlineLevel="0" r="73">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t>205/55R16</t>
+          <t>205/50R17</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>AMINE</t>
+          <t>CONTINENTAL</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
-          <t>AM205/55R16</t>
+          <t>CT205/50R17</t>
         </is>
       </c>
       <c r="D73" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E73" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F73" s="0">
         <v>0</v>
@@ -2693,7 +2693,7 @@
         <v>0</v>
       </c>
       <c r="H73" s="1">
-        <v>240</v>
+        <v>450</v>
       </c>
     </row>
     <row outlineLevel="0" r="74">
@@ -2704,19 +2704,19 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>DOUBLESTAR</t>
+          <t>AMINE</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
         <is>
-          <t>DS205/55R16</t>
+          <t>AM205/55R16</t>
         </is>
       </c>
       <c r="D74" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E74" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F74" s="0">
         <v>0</v>
@@ -2725,7 +2725,7 @@
         <v>0</v>
       </c>
       <c r="H74" s="1">
-        <v>230</v>
+        <v>240</v>
       </c>
     </row>
     <row outlineLevel="0" r="75">
@@ -2736,28 +2736,28 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>FULDA</t>
+          <t>DOUBLESTAR</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
         <is>
-          <t>FL205/55R16</t>
+          <t>DS205/55R16</t>
         </is>
       </c>
       <c r="D75" s="0">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="E75" s="0">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F75" s="0">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="G75" s="0">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H75" s="1">
-        <v>250</v>
+        <v>230</v>
       </c>
     </row>
     <row outlineLevel="0" r="76">
@@ -2768,25 +2768,25 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>GOODRIDE</t>
+          <t>FULDA</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
         <is>
-          <t>GR205/55R16</t>
+          <t>FL205/55R16</t>
         </is>
       </c>
       <c r="D76" s="0">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="E76" s="0">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F76" s="0">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="G76" s="0">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H76" s="1">
         <v>250</v>
@@ -2800,28 +2800,28 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>GOODRIDE</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
         <is>
-          <t>GD205/55R16</t>
+          <t>GR205/55R16</t>
         </is>
       </c>
       <c r="D77" s="0">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E77" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F77" s="0">
         <v>0</v>
       </c>
       <c r="G77" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H77" s="1">
-        <v>280</v>
+        <v>250</v>
       </c>
     </row>
     <row outlineLevel="0" r="78">
@@ -2832,28 +2832,28 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
         <is>
-          <t>HK205/55R16</t>
+          <t>GD205/55R16</t>
         </is>
       </c>
       <c r="D78" s="0">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E78" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F78" s="0">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G78" s="0">
         <v>4</v>
       </c>
       <c r="H78" s="1">
-        <v>260</v>
+        <v>280</v>
       </c>
     </row>
     <row outlineLevel="0" r="79">
@@ -2864,48 +2864,48 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
         <is>
-          <t>RD205/55R16</t>
+          <t>HK205/55R16</t>
         </is>
       </c>
       <c r="D79" s="0">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="E79" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F79" s="0">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G79" s="0">
         <v>4</v>
       </c>
       <c r="H79" s="1">
-        <v>230</v>
+        <v>260</v>
       </c>
     </row>
     <row outlineLevel="0" r="80">
       <c r="A80" s="0" t="inlineStr">
         <is>
-          <t>205/55R16RF</t>
+          <t>205/55R16</t>
         </is>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
         <is>
-          <t>GD205/55R16RF</t>
+          <t>RD205/55R16</t>
         </is>
       </c>
       <c r="D80" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E80" s="0">
         <v>0</v>
@@ -2914,16 +2914,16 @@
         <v>0</v>
       </c>
       <c r="G80" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H80" s="1">
-        <v>480</v>
+        <v>230</v>
       </c>
     </row>
     <row outlineLevel="0" r="81">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t>205/55R17</t>
+          <t>205/55R16RF</t>
         </is>
       </c>
       <c r="B81" s="0" t="inlineStr">
@@ -2933,23 +2933,23 @@
       </c>
       <c r="C81" s="0" t="inlineStr">
         <is>
-          <t>GD205/55R17</t>
+          <t>GD205/55R16RF</t>
         </is>
       </c>
       <c r="D81" s="0">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E81" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F81" s="0">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G81" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H81" s="1">
-        <v>450</v>
+        <v>480</v>
       </c>
     </row>
     <row outlineLevel="0" r="82">
@@ -2960,51 +2960,51 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>NEXEN</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
         <is>
-          <t>NX205/55R17</t>
+          <t>GD205/55R17</t>
         </is>
       </c>
       <c r="D82" s="0">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E82" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F82" s="0">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G82" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H82" s="1">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row outlineLevel="0" r="83">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t>205/60R16</t>
+          <t>205/55R17</t>
         </is>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>DUNLOP</t>
+          <t>NEXEN</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
         <is>
-          <t>DL205/60R16</t>
+          <t>NX205/55R17</t>
         </is>
       </c>
       <c r="D83" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E83" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F83" s="0">
         <v>0</v>
@@ -3013,7 +3013,7 @@
         <v>0</v>
       </c>
       <c r="H83" s="1">
-        <v>330</v>
+        <v>400</v>
       </c>
     </row>
     <row outlineLevel="0" r="84">
@@ -3024,28 +3024,28 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>DUNLOP</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
         <is>
-          <t>GD205/60R16</t>
+          <t>DL205/60R16</t>
         </is>
       </c>
       <c r="D84" s="0">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E84" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F84" s="0">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G84" s="0">
         <v>0</v>
       </c>
       <c r="H84" s="1">
-        <v>380</v>
+        <v>330</v>
       </c>
     </row>
     <row outlineLevel="0" r="85">
@@ -3056,28 +3056,28 @@
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
         <is>
-          <t>HK205/60R16</t>
+          <t>GD205/60R16</t>
         </is>
       </c>
       <c r="D85" s="0">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E85" s="0">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F85" s="0">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G85" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H85" s="1">
-        <v>300</v>
+        <v>380</v>
       </c>
     </row>
     <row outlineLevel="0" r="86">
@@ -3088,25 +3088,25 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>LUFEN</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
         <is>
-          <t>LF205/60R16</t>
+          <t>HK205/60R16</t>
         </is>
       </c>
       <c r="D86" s="0">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E86" s="0">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F86" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G86" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H86" s="1">
         <v>300</v>
@@ -3115,24 +3115,24 @@
     <row outlineLevel="0" r="87">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t>205/65R15</t>
+          <t>205/60R16</t>
         </is>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>LUFEN</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
         <is>
-          <t>HK205/65R15</t>
+          <t>LF205/60R16</t>
         </is>
       </c>
       <c r="D87" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E87" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F87" s="0">
         <v>0</v>
@@ -3141,30 +3141,30 @@
         <v>0</v>
       </c>
       <c r="H87" s="1">
-        <v>270</v>
+        <v>300</v>
       </c>
     </row>
     <row outlineLevel="0" r="88">
       <c r="A88" s="0" t="inlineStr">
         <is>
-          <t>205/65R16</t>
+          <t>205/65R15</t>
         </is>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>BRIDGESTONE</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
         <is>
-          <t>BR205/65R16</t>
+          <t>HK205/65R15</t>
         </is>
       </c>
       <c r="D88" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E88" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F88" s="0">
         <v>0</v>
@@ -3173,7 +3173,7 @@
         <v>0</v>
       </c>
       <c r="H88" s="1">
-        <v>420</v>
+        <v>270</v>
       </c>
     </row>
     <row outlineLevel="0" r="89">
@@ -3184,19 +3184,19 @@
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>BRIDGESTONE</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
         <is>
-          <t>HK205/65R16</t>
+          <t>BR205/65R16</t>
         </is>
       </c>
       <c r="D89" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E89" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F89" s="0">
         <v>0</v>
@@ -3205,39 +3205,39 @@
         <v>0</v>
       </c>
       <c r="H89" s="1">
-        <v>380</v>
+        <v>420</v>
       </c>
     </row>
     <row outlineLevel="0" r="90">
       <c r="A90" s="0" t="inlineStr">
         <is>
-          <t>215/40R18</t>
+          <t>205/65R16</t>
         </is>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
         <is>
-          <t>GD215/40R18</t>
+          <t>HK205/65R16</t>
         </is>
       </c>
       <c r="D90" s="0">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E90" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F90" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G90" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H90" s="1">
-        <v>600</v>
+        <v>380</v>
       </c>
     </row>
     <row outlineLevel="0" r="91">
@@ -3248,44 +3248,44 @@
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
         <is>
-          <t>HK215/40R18</t>
+          <t>GD215/40R18</t>
         </is>
       </c>
       <c r="D91" s="0">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E91" s="0">
         <v>4</v>
       </c>
       <c r="F91" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G91" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H91" s="1">
-        <v>490</v>
+        <v>600</v>
       </c>
     </row>
     <row outlineLevel="0" r="92">
       <c r="A92" s="0" t="inlineStr">
         <is>
-          <t>215/45R16</t>
+          <t>215/40R18</t>
         </is>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
         <is>
-          <t>GD215/45R16</t>
+          <t>HK215/40R18</t>
         </is>
       </c>
       <c r="D92" s="0">
@@ -3301,13 +3301,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="1">
-        <v>450</v>
+        <v>490</v>
       </c>
     </row>
     <row outlineLevel="0" r="93">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t>215/45R17</t>
+          <t>215/45R16</t>
         </is>
       </c>
       <c r="B93" s="0" t="inlineStr">
@@ -3317,14 +3317,14 @@
       </c>
       <c r="C93" s="0" t="inlineStr">
         <is>
-          <t>GD215/45R17</t>
+          <t>GD215/45R16</t>
         </is>
       </c>
       <c r="D93" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E93" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F93" s="0">
         <v>0</v>
@@ -3333,7 +3333,7 @@
         <v>0</v>
       </c>
       <c r="H93" s="1">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row outlineLevel="0" r="94">
@@ -3344,25 +3344,25 @@
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
         <is>
-          <t>HK215/45R17</t>
+          <t>GD215/45R17</t>
         </is>
       </c>
       <c r="D94" s="0">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E94" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F94" s="0">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G94" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H94" s="1">
         <v>400</v>
@@ -3376,28 +3376,28 @@
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>IRIS</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
         <is>
-          <t>IR215/45R17</t>
+          <t>HK215/45R17</t>
         </is>
       </c>
       <c r="D95" s="0">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="E95" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F95" s="0">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G95" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H95" s="1">
-        <v>300</v>
+        <v>400</v>
       </c>
     </row>
     <row outlineLevel="0" r="96">
@@ -3408,28 +3408,28 @@
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>LUFEN</t>
+          <t>IRIS</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
         <is>
-          <t>LF215/45R17</t>
+          <t>IR215/45R17</t>
         </is>
       </c>
       <c r="D96" s="0">
         <v>1</v>
       </c>
       <c r="E96" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F96" s="0">
         <v>0</v>
       </c>
       <c r="G96" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H96" s="1">
-        <v>350</v>
+        <v>300</v>
       </c>
     </row>
     <row outlineLevel="0" r="97">
@@ -3440,83 +3440,83 @@
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>NEXEN</t>
+          <t>LUFEN</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
         <is>
-          <t>NX215/45R17</t>
+          <t>LF215/45R17</t>
         </is>
       </c>
       <c r="D97" s="0">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E97" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F97" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G97" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H97" s="1">
-        <v>380</v>
+        <v>350</v>
       </c>
     </row>
     <row outlineLevel="0" r="98">
       <c r="A98" s="0" t="inlineStr">
         <is>
-          <t>215/45R18</t>
+          <t>215/45R17</t>
         </is>
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>NEXEN</t>
         </is>
       </c>
       <c r="C98" s="0" t="inlineStr">
         <is>
-          <t>GD215/45R18</t>
+          <t>NX215/45R17</t>
         </is>
       </c>
       <c r="D98" s="0">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E98" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F98" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G98" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H98" s="1">
-        <v>550</v>
+        <v>380</v>
       </c>
     </row>
     <row outlineLevel="0" r="99">
       <c r="A99" s="0" t="inlineStr">
         <is>
-          <t>215/50R17</t>
+          <t>215/45R18</t>
         </is>
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>BRIDGESTONE</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C99" s="0" t="inlineStr">
         <is>
-          <t>BR215/50R17</t>
+          <t>GD215/45R18</t>
         </is>
       </c>
       <c r="D99" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E99" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F99" s="0">
         <v>0</v>
@@ -3525,7 +3525,7 @@
         <v>0</v>
       </c>
       <c r="H99" s="1">
-        <v>450</v>
+        <v>550</v>
       </c>
     </row>
     <row outlineLevel="0" r="100">
@@ -3536,28 +3536,28 @@
       </c>
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>BRIDGESTONE</t>
         </is>
       </c>
       <c r="C100" s="0" t="inlineStr">
         <is>
-          <t>GD215/50R17</t>
+          <t>BR215/50R17</t>
         </is>
       </c>
       <c r="D100" s="0">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E100" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F100" s="0">
         <v>0</v>
       </c>
       <c r="G100" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H100" s="1">
-        <v>470</v>
+        <v>450</v>
       </c>
     </row>
     <row outlineLevel="0" r="101">
@@ -3568,28 +3568,28 @@
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C101" s="0" t="inlineStr">
         <is>
-          <t>HK215/50R17</t>
+          <t>GD215/50R17</t>
         </is>
       </c>
       <c r="D101" s="0">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E101" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F101" s="0">
         <v>0</v>
       </c>
       <c r="G101" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H101" s="1">
-        <v>400</v>
+        <v>470</v>
       </c>
     </row>
     <row outlineLevel="0" r="102">
@@ -3600,19 +3600,19 @@
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t>LUFEN</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C102" s="0" t="inlineStr">
         <is>
-          <t>LF215/50R17</t>
+          <t>HK215/50R17</t>
         </is>
       </c>
       <c r="D102" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E102" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F102" s="0">
         <v>0</v>
@@ -3621,30 +3621,30 @@
         <v>0</v>
       </c>
       <c r="H102" s="1">
-        <v>420</v>
+        <v>400</v>
       </c>
     </row>
     <row outlineLevel="0" r="103">
       <c r="A103" s="0" t="inlineStr">
         <is>
-          <t>215/50R18</t>
+          <t>215/50R17</t>
         </is>
       </c>
       <c r="B103" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>LUFEN</t>
         </is>
       </c>
       <c r="C103" s="0" t="inlineStr">
         <is>
-          <t>GD215/50R18</t>
+          <t>LF215/50R17</t>
         </is>
       </c>
       <c r="D103" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E103" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F103" s="0">
         <v>0</v>
@@ -3653,13 +3653,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="1">
-        <v>600</v>
+        <v>420</v>
       </c>
     </row>
     <row outlineLevel="0" r="104">
       <c r="A104" s="0" t="inlineStr">
         <is>
-          <t>215/55R16</t>
+          <t>215/50R18</t>
         </is>
       </c>
       <c r="B104" s="0" t="inlineStr">
@@ -3669,14 +3669,14 @@
       </c>
       <c r="C104" s="0" t="inlineStr">
         <is>
-          <t>GD215/55R16</t>
+          <t>GD215/50R18</t>
         </is>
       </c>
       <c r="D104" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E104" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F104" s="0">
         <v>0</v>
@@ -3685,7 +3685,7 @@
         <v>0</v>
       </c>
       <c r="H104" s="1">
-        <v>440</v>
+        <v>600</v>
       </c>
     </row>
     <row outlineLevel="0" r="105">
@@ -3696,12 +3696,12 @@
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t>LUFEN</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C105" s="0" t="inlineStr">
         <is>
-          <t>LF215/55R16</t>
+          <t>GD215/55R16</t>
         </is>
       </c>
       <c r="D105" s="0">
@@ -3717,23 +3717,23 @@
         <v>0</v>
       </c>
       <c r="H105" s="1">
-        <v>350</v>
+        <v>440</v>
       </c>
     </row>
     <row outlineLevel="0" r="106">
       <c r="A106" s="0" t="inlineStr">
         <is>
-          <t>215/55R17</t>
+          <t>215/55R16</t>
         </is>
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t>BRIDGESTONE</t>
+          <t>LUFEN</t>
         </is>
       </c>
       <c r="C106" s="0" t="inlineStr">
         <is>
-          <t>BR215/55R17</t>
+          <t>LF215/55R16</t>
         </is>
       </c>
       <c r="D106" s="0">
@@ -3749,7 +3749,7 @@
         <v>0</v>
       </c>
       <c r="H106" s="1">
-        <v>480</v>
+        <v>350</v>
       </c>
     </row>
     <row outlineLevel="0" r="107">
@@ -3760,19 +3760,19 @@
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>BRIDGESTONE</t>
         </is>
       </c>
       <c r="C107" s="0" t="inlineStr">
         <is>
-          <t>HK215/55R17</t>
+          <t>BR215/55R17</t>
         </is>
       </c>
       <c r="D107" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E107" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F107" s="0">
         <v>0</v>
@@ -3781,23 +3781,23 @@
         <v>0</v>
       </c>
       <c r="H107" s="1">
-        <v>420</v>
+        <v>480</v>
       </c>
     </row>
     <row outlineLevel="0" r="108">
       <c r="A108" s="0" t="inlineStr">
         <is>
-          <t>215/55R18</t>
+          <t>215/55R17</t>
         </is>
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C108" s="0" t="inlineStr">
         <is>
-          <t>GD215/55R18</t>
+          <t>HK215/55R17</t>
         </is>
       </c>
       <c r="D108" s="0">
@@ -3813,23 +3813,23 @@
         <v>0</v>
       </c>
       <c r="H108" s="1">
-        <v>580</v>
+        <v>420</v>
       </c>
     </row>
     <row outlineLevel="0" r="109">
       <c r="A109" s="0" t="inlineStr">
         <is>
-          <t>215/60R16</t>
+          <t>215/55R18</t>
         </is>
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t>BRIDGESTONE</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C109" s="0" t="inlineStr">
         <is>
-          <t>BR215/60R16</t>
+          <t>GD215/55R18</t>
         </is>
       </c>
       <c r="D109" s="0">
@@ -3845,7 +3845,7 @@
         <v>0</v>
       </c>
       <c r="H109" s="1">
-        <v>350</v>
+        <v>580</v>
       </c>
     </row>
     <row outlineLevel="0" r="110">
@@ -3856,25 +3856,25 @@
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t>DUNLOP</t>
+          <t>BRIDGESTONE</t>
         </is>
       </c>
       <c r="C110" s="0" t="inlineStr">
         <is>
-          <t>DL215/60R16</t>
+          <t>BR215/60R16</t>
         </is>
       </c>
       <c r="D110" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E110" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F110" s="0">
         <v>0</v>
       </c>
       <c r="G110" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H110" s="1">
         <v>350</v>
@@ -3888,28 +3888,28 @@
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>DUNLOP</t>
         </is>
       </c>
       <c r="C111" s="0" t="inlineStr">
         <is>
-          <t>HK215/60R16</t>
+          <t>DL215/60R16</t>
         </is>
       </c>
       <c r="D111" s="0">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E111" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F111" s="0">
         <v>0</v>
       </c>
       <c r="G111" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H111" s="1">
-        <v>330</v>
+        <v>350</v>
       </c>
     </row>
     <row outlineLevel="0" r="112">
@@ -3920,25 +3920,25 @@
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t>NEXEN</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C112" s="0" t="inlineStr">
         <is>
-          <t>NX215/60R16</t>
+          <t>HK215/60R16</t>
         </is>
       </c>
       <c r="D112" s="0">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E112" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F112" s="0">
         <v>0</v>
       </c>
       <c r="G112" s="0">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H112" s="1">
         <v>330</v>
@@ -3947,65 +3947,65 @@
     <row outlineLevel="0" r="113">
       <c r="A113" s="0" t="inlineStr">
         <is>
-          <t>215/60R17</t>
+          <t>215/60R16</t>
         </is>
       </c>
       <c r="B113" s="0" t="inlineStr">
         <is>
-          <t>RADIAL</t>
+          <t>NEXEN</t>
         </is>
       </c>
       <c r="C113" s="0" t="inlineStr">
         <is>
-          <t>RD215/60R17</t>
+          <t>NX215/60R16</t>
         </is>
       </c>
       <c r="D113" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E113" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F113" s="0">
         <v>0</v>
       </c>
       <c r="G113" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H113" s="1">
-        <v>300</v>
+        <v>330</v>
       </c>
     </row>
     <row outlineLevel="0" r="114">
       <c r="A114" s="0" t="inlineStr">
         <is>
-          <t>215/65R16</t>
+          <t>215/60R17</t>
         </is>
       </c>
       <c r="B114" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>RADIAL</t>
         </is>
       </c>
       <c r="C114" s="0" t="inlineStr">
         <is>
-          <t>GD215/65R16</t>
+          <t>RD215/60R17</t>
         </is>
       </c>
       <c r="D114" s="0">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E114" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F114" s="0">
         <v>0</v>
       </c>
       <c r="G114" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H114" s="1">
-        <v>380</v>
+        <v>300</v>
       </c>
     </row>
     <row outlineLevel="0" r="115">
@@ -4016,83 +4016,83 @@
       </c>
       <c r="B115" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C115" s="0" t="inlineStr">
         <is>
-          <t>HK215/65R16</t>
+          <t>GD215/65R16</t>
         </is>
       </c>
       <c r="D115" s="0">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E115" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F115" s="0">
         <v>0</v>
       </c>
       <c r="G115" s="0">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H115" s="1">
-        <v>330</v>
+        <v>380</v>
       </c>
     </row>
     <row outlineLevel="0" r="116">
       <c r="A116" s="0" t="inlineStr">
         <is>
-          <t>215/65R17</t>
+          <t>215/65R16</t>
         </is>
       </c>
       <c r="B116" s="0" t="inlineStr">
         <is>
-          <t>MICHELIN</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C116" s="0" t="inlineStr">
         <is>
-          <t>MC215/65R17</t>
+          <t>HK215/65R16</t>
         </is>
       </c>
       <c r="D116" s="0">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E116" s="0">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F116" s="0">
         <v>0</v>
       </c>
       <c r="G116" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H116" s="1">
-        <v>600</v>
+        <v>330</v>
       </c>
     </row>
     <row outlineLevel="0" r="117">
       <c r="A117" s="0" t="inlineStr">
         <is>
-          <t>225/40R18</t>
+          <t>215/65R17</t>
         </is>
       </c>
       <c r="B117" s="0" t="inlineStr">
         <is>
-          <t>BARUM</t>
+          <t>MICHELIN</t>
         </is>
       </c>
       <c r="C117" s="0" t="inlineStr">
         <is>
-          <t>BM225/40R18</t>
+          <t>MC215/65R17</t>
         </is>
       </c>
       <c r="D117" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E117" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F117" s="0">
         <v>0</v>
@@ -4101,7 +4101,7 @@
         <v>0</v>
       </c>
       <c r="H117" s="1">
-        <v>420</v>
+        <v>600</v>
       </c>
     </row>
     <row outlineLevel="0" r="118">
@@ -4112,28 +4112,28 @@
       </c>
       <c r="B118" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>BARUM</t>
         </is>
       </c>
       <c r="C118" s="0" t="inlineStr">
         <is>
-          <t>GD225/40R18</t>
+          <t>BM225/40R18</t>
         </is>
       </c>
       <c r="D118" s="0">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E118" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F118" s="0">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G118" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H118" s="1">
-        <v>480</v>
+        <v>420</v>
       </c>
     </row>
     <row outlineLevel="0" r="119">
@@ -4144,28 +4144,28 @@
       </c>
       <c r="B119" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C119" s="0" t="inlineStr">
         <is>
-          <t>HK225/40R18</t>
+          <t>GD225/40R18</t>
         </is>
       </c>
       <c r="D119" s="0">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E119" s="0">
         <v>4</v>
       </c>
       <c r="F119" s="0">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G119" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H119" s="1">
-        <v>450</v>
+        <v>480</v>
       </c>
     </row>
     <row outlineLevel="0" r="120">
@@ -4176,28 +4176,28 @@
       </c>
       <c r="B120" s="0" t="inlineStr">
         <is>
-          <t>LASSA</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C120" s="0" t="inlineStr">
         <is>
-          <t>LS225/40R18</t>
+          <t>HK225/40R18</t>
         </is>
       </c>
       <c r="D120" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E120" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F120" s="0">
         <v>0</v>
       </c>
       <c r="G120" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H120" s="1">
-        <v>330</v>
+        <v>450</v>
       </c>
     </row>
     <row outlineLevel="0" r="121">
@@ -4208,28 +4208,28 @@
       </c>
       <c r="B121" s="0" t="inlineStr">
         <is>
-          <t>NEXEN</t>
+          <t>LASSA</t>
         </is>
       </c>
       <c r="C121" s="0" t="inlineStr">
         <is>
-          <t>NX225/40R18</t>
+          <t>LS225/40R18</t>
         </is>
       </c>
       <c r="D121" s="0">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E121" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F121" s="0">
         <v>0</v>
       </c>
       <c r="G121" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H121" s="1">
-        <v>400</v>
+        <v>330</v>
       </c>
     </row>
     <row outlineLevel="0" r="122">
@@ -4240,19 +4240,19 @@
       </c>
       <c r="B122" s="0" t="inlineStr">
         <is>
-          <t>SEMPERIT</t>
+          <t>NEXEN</t>
         </is>
       </c>
       <c r="C122" s="0" t="inlineStr">
         <is>
-          <t>SP225/40R18</t>
+          <t>NX225/40R18</t>
         </is>
       </c>
       <c r="D122" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E122" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F122" s="0">
         <v>0</v>
@@ -4261,30 +4261,30 @@
         <v>0</v>
       </c>
       <c r="H122" s="1">
-        <v>450</v>
+        <v>400</v>
       </c>
     </row>
     <row outlineLevel="0" r="123">
       <c r="A123" s="0" t="inlineStr">
         <is>
-          <t>225/40R18RF</t>
+          <t>225/40R18</t>
         </is>
       </c>
       <c r="B123" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>SEMPERIT</t>
         </is>
       </c>
       <c r="C123" s="0" t="inlineStr">
         <is>
-          <t>GD225/40R18RF</t>
+          <t>SP225/40R18</t>
         </is>
       </c>
       <c r="D123" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E123" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F123" s="0">
         <v>0</v>
@@ -4293,30 +4293,30 @@
         <v>0</v>
       </c>
       <c r="H123" s="1">
-        <v>590</v>
+        <v>450</v>
       </c>
     </row>
     <row outlineLevel="0" r="124">
       <c r="A124" s="0" t="inlineStr">
         <is>
-          <t>225/45R17</t>
+          <t>225/40R18RF</t>
         </is>
       </c>
       <c r="B124" s="0" t="inlineStr">
         <is>
-          <t>CONTINENTAL</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C124" s="0" t="inlineStr">
         <is>
-          <t>CT225/45R17</t>
+          <t>GD225/40R18RF</t>
         </is>
       </c>
       <c r="D124" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E124" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F124" s="0">
         <v>0</v>
@@ -4325,7 +4325,7 @@
         <v>0</v>
       </c>
       <c r="H124" s="1">
-        <v>400</v>
+        <v>590</v>
       </c>
     </row>
     <row outlineLevel="0" r="125">
@@ -4336,28 +4336,28 @@
       </c>
       <c r="B125" s="0" t="inlineStr">
         <is>
-          <t>FULDA</t>
+          <t>CONTINENTAL</t>
         </is>
       </c>
       <c r="C125" s="0" t="inlineStr">
         <is>
-          <t>FL225/45R17</t>
+          <t>CT225/45R17</t>
         </is>
       </c>
       <c r="D125" s="0">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="E125" s="0">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F125" s="0">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G125" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H125" s="1">
-        <v>350</v>
+        <v>400</v>
       </c>
     </row>
     <row outlineLevel="0" r="126">
@@ -4368,28 +4368,28 @@
       </c>
       <c r="B126" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>FULDA</t>
         </is>
       </c>
       <c r="C126" s="0" t="inlineStr">
         <is>
-          <t>GD225/45R17</t>
+          <t>FL225/45R17</t>
         </is>
       </c>
       <c r="D126" s="0">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E126" s="0">
         <v>6</v>
       </c>
       <c r="F126" s="0">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G126" s="0">
         <v>4</v>
       </c>
       <c r="H126" s="1">
-        <v>380</v>
+        <v>350</v>
       </c>
     </row>
     <row outlineLevel="0" r="127">
@@ -4400,60 +4400,60 @@
       </c>
       <c r="B127" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C127" s="0" t="inlineStr">
         <is>
-          <t>HK225/45R17</t>
+          <t>GD225/45R17</t>
         </is>
       </c>
       <c r="D127" s="0">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="E127" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F127" s="0">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G127" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H127" s="1">
-        <v>350</v>
+        <v>380</v>
       </c>
     </row>
     <row outlineLevel="0" r="128">
       <c r="A128" s="0" t="inlineStr">
         <is>
-          <t>225/45R18</t>
+          <t>225/45R17</t>
         </is>
       </c>
       <c r="B128" s="0" t="inlineStr">
         <is>
-          <t>DUNLOP</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C128" s="0" t="inlineStr">
         <is>
-          <t>DL225/45R18</t>
+          <t>HK225/45R17</t>
         </is>
       </c>
       <c r="D128" s="0">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E128" s="0">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F128" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G128" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H128" s="1">
-        <v>500</v>
+        <v>350</v>
       </c>
     </row>
     <row outlineLevel="0" r="129">
@@ -4464,28 +4464,28 @@
       </c>
       <c r="B129" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>DUNLOP</t>
         </is>
       </c>
       <c r="C129" s="0" t="inlineStr">
         <is>
-          <t>GD225/45R18</t>
+          <t>DL225/45R18</t>
         </is>
       </c>
       <c r="D129" s="0">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E129" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F129" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G129" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H129" s="1">
-        <v>550</v>
+        <v>500</v>
       </c>
     </row>
     <row outlineLevel="0" r="130">
@@ -4496,28 +4496,28 @@
       </c>
       <c r="B130" s="0" t="inlineStr">
         <is>
-          <t>HANKOOK</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C130" s="0" t="inlineStr">
         <is>
-          <t>HK225/45R18</t>
+          <t>GD225/45R18</t>
         </is>
       </c>
       <c r="D130" s="0">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E130" s="0">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F130" s="0">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G130" s="0">
         <v>0</v>
       </c>
       <c r="H130" s="1">
-        <v>450</v>
+        <v>550</v>
       </c>
     </row>
     <row outlineLevel="0" r="131">
@@ -4528,19 +4528,19 @@
       </c>
       <c r="B131" s="0" t="inlineStr">
         <is>
-          <t>LUFEN</t>
+          <t>HANKOOK</t>
         </is>
       </c>
       <c r="C131" s="0" t="inlineStr">
         <is>
-          <t>LF225/45R18</t>
+          <t>HK225/45R18</t>
         </is>
       </c>
       <c r="D131" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E131" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F131" s="0">
         <v>0</v>
@@ -4549,71 +4549,71 @@
         <v>0</v>
       </c>
       <c r="H131" s="1">
-        <v>420</v>
+        <v>450</v>
       </c>
     </row>
     <row outlineLevel="0" r="132">
       <c r="A132" s="0" t="inlineStr">
         <is>
-          <t>225/45R18RF</t>
+          <t>225/45R18</t>
         </is>
       </c>
       <c r="B132" s="0" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>LUFEN</t>
         </is>
       </c>
       <c r="C132" s="0" t="inlineStr">
         <is>
-          <t>GD225/45R18RF</t>
+          <t>LF225/45R18</t>
         </is>
       </c>
       <c r="D132" s="0">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E132" s="0">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F132" s="0">
         <v>0</v>
       </c>
       <c r="G132" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H132" s="1">
-        <v>720</v>
+        <v>420</v>
       </c>
     </row>
     <row outlineLevel="0" r="133">
       <c r="A133" s="0" t="inlineStr">
         <is>
-          <t>225/45R19</t>
+          <t>225/45R18RF</t>
         </is>
       </c>
       <c r="B133" s="0" t="inlineStr">
         <is>
-          <t>CONTINENTAL</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="C133" s="0" t="inlineStr">
         <is>
-          <t>CT225/45R19</t>
+          <t>GD225/45R18RF</t>
         </is>
       </c>
       <c r="D133" s="0">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E133" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F133" s="0">
         <v>0</v>
       </c>
       <c r="G133" s="0">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H133" s="1">
-        <v>780</v>
+        <v>720</v>
       </c>
     </row>
     <row outlineLevel="0" r="134">
@@ -4624,12 +4624,12 @@
       </c>
       <c r="B134" s="0" t="inlineStr">
         <is>
-          <t>LASSA</t>
+          <t>CONTINENTAL</t>
         </is>
       </c>
       <c r="C134" s="0" t="inlineStr">
         <is>
-          <t>LS225/45R19</t>
+          <t>CT225/45R19</t>
         </is>
       </c>
       <c r="D134" s="0">
@@ -4645,7 +4645,7 @@
         <v>0</v>
       </c>
       <c r="H134" s="1">
-        <v>520</v>
+        <v>780</v>
       </c>
     </row>
     <row outlineLevel="0" r="135">
@@ -4697,10 +4697,10 @@
         </is>
       </c>
       <c r="D136" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E136" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F136" s="0">
         <v>8</v>
@@ -6553,13 +6553,13 @@
         </is>
       </c>
       <c r="D194" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E194" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F194" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G194" s="0">
         <v>0</v>

</xml_diff>